<commit_message>
feat: improve LR dashboard filters, PAN styling, and locations
Style PAN cells left-aligned in brand orange, add Mahalaxmi Industries to consignor/consignee options, and exclude cancelled LRs from LR This Month views, exports, and month-scoped cancelled counts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/LR MASTER COPY.xlsx
+++ b/LR MASTER COPY.xlsx
@@ -62,6 +62,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <color rgb="FFFF3300"/>
+        <sz val="13"/>
+        <rFont val="Calibri"/>
+      </rPr>
       <t xml:space="preserve">E-way Bill : </t>
     </r>
     <r>
@@ -76,6 +81,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <color rgb="FFFF3300"/>
+        <sz val="13"/>
+        <rFont val="Calibri"/>
+      </rPr>
       <t xml:space="preserve">PAN : </t>
     </r>
     <r>
@@ -191,12 +201,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFFF3300"/>
+      <sz val="13"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -524,195 +539,195 @@
   </cellStyleXfs>
   <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+      <alignment horizontal="left" indent="4"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>

</xml_diff>